<commit_message>
Vendor-style test upload: D-range sets, pictures, optional option E, richer question details
- Word: Topic / Q.n) / a)-e) / Answer / Explanation; D.51-55) groups RC and DILR sets; pictures upload to the media table
- Option E only where a question has five options (bank form shows it on demand)
- Excel details: Type, Difficulty Level (Very Easy-Very Hard), Concepts, Source, Subject paths fill section > topic > subtopic
- Guru sees the student's weakest topics with unseen bank question counts
- Indexes for topic/level, subtopic and tag lookups; new templates

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HobNgf1JPqeUaeRZMhfYbX
</commit_message>
<xml_diff>
--- a/portal/public/question-details-template.xlsx
+++ b/portal/public/question-details-template.xlsx
@@ -44,7 +44,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3A8A"/>
+        <fgColor rgb="001E40AF"/>
       </patternFill>
     </fill>
   </fills>
@@ -63,7 +63,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -140,6 +140,76 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>DE Educare</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Same test name as the "Test:" line in Word. Can stay blank if the file has one test.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Fill if question numbers restart in each section.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Same number as in Word (Q.1) → 1).</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional if the Word file has Topic: lines (Word wins). Pick from the Topics sheet.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>The finer skill inside the topic, e.g. Successive discounts. Guru and practice sets use it.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Single (one answer), Multiple (several answers) or Numeric (type-in). Blank: worked out from the answer.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Very Easy, Easy, Medium, Hard or Very Hard.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>Time a well-prepared student should take, in seconds. Used in time analysis.</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>Comma-separated concepts or question patterns, e.g. ratio, weighted average. Guru uses them to find similar questions.</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>Original, or the paper, e.g. CAT 2023 Slot 2 (previous-year questions).</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <t>Only if the Word file has no Answer: line. a, or a,c for Multiple, or a number.</t>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <t>English, Hindi or Both.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -431,21 +501,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -461,7 +534,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Q No</t>
+          <t>Question Number</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -476,37 +549,52 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Difficulty</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Difficulty Level</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Ideal time (sec)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Marks if correct</t>
-        </is>
-      </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Negative marks</t>
+          <t>Marks</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Tags</t>
+          <t>Negative Marks</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>Concepts</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Image link</t>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Correct Answer(s)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Solution video</t>
         </is>
       </c>
     </row>
@@ -536,29 +624,40 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>120</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>3</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>1</v>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>rc</t>
-        </is>
-      </c>
       <c r="K2" t="inlineStr">
         <is>
+          <t>main idea, tone</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
           <t>Original</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -586,29 +685,40 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>Hard</t>
         </is>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>150</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>3</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>1</v>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>rc</t>
-        </is>
-      </c>
       <c r="K3" t="inlineStr">
         <is>
+          <t>inference</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
           <t>Original</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -618,47 +728,58 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>QA</t>
+          <t>VARC</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Percentages</t>
+          <t>Para Jumbles</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Successive change</t>
+          <t>Four-sentence jumble</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>60</v>
+          <t>Numeric</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Very Hard</t>
+        </is>
       </c>
       <c r="H4" t="n">
+        <v>120</v>
+      </c>
+      <c r="I4" t="n">
         <v>3</v>
       </c>
-      <c r="I4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>percent</t>
-        </is>
+      <c r="J4" t="n">
+        <v>0</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Original</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
+          <t>opening sentence, linkers</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>CAT 2023 Slot 2</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -672,7 +793,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -681,39 +802,50 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Basics</t>
+          <t>Successive change</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>Easy</t>
         </is>
       </c>
-      <c r="G5" t="n">
-        <v>45</v>
-      </c>
       <c r="H5" t="n">
+        <v>60</v>
+      </c>
+      <c r="I5" t="n">
         <v>3</v>
       </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>tita</t>
-        </is>
+      <c r="J5" t="n">
+        <v>1</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
+          <t>multiplying factors</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
           <t>Original</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAT Mock 2</t>
+          <t>CAT Mock 1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -722,47 +854,187 @@
         </is>
       </c>
       <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Percentages</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Percent of a number</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Numeric</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>30</v>
+      </c>
+      <c r="I6" t="n">
+        <v>3</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Bank PO Mock 1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
         <v>1</v>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Time, Speed &amp; Distance</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Relative speed</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Data Interpretation</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Bar graph</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G6" t="n">
-        <v>90</v>
-      </c>
-      <c r="H6" t="n">
-        <v>3</v>
-      </c>
-      <c r="I6" t="n">
+      <c r="H7" t="n">
+        <v>60</v>
+      </c>
+      <c r="I7" t="n">
         <v>1</v>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>CAT 2024 Slot 1</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
+      <c r="J7" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>difference, ranking</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Bank PO Mock 1</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Data Interpretation</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Bar graph</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>60</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="F2:F2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Easy,Medium,Hard"</formula1>
+  <dataValidations count="3">
+    <dataValidation sqref="F2:F5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Single,Multiple,Numeric"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Very Easy,Easy,Medium,Hard,Very Hard"</formula1>
+    </dataValidation>
+    <dataValidation sqref="N2:N5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"English,Hindi,Both"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -775,10 +1047,10 @@
   <dimension ref="A1:D73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2398,7 +2670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -2407,42 +2679,56 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>One row per question in the Word file. Test, Section and Q No must match the Word file (same test name, same section name, same question number).</t>
+          <t>One row per question in the Word file. Test, Section and Question Number must match the Word file.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>If question numbers restart in each section, fill Section. If they run through the whole test, Section can stay blank.</t>
+          <t>If question numbers restart in each section, fill Section. If they run through the whole test (like Q.51 … Q.55), Section can stay blank.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Topic: pick from the Topics sheet so reports and the auto test builder group questions correctly. A new topic is created if you type one that is not in the list.</t>
+          <t>Every column helps the question bank: Topic and Subtopic drive topic reports, SWOT and practice sets; Difficulty and Ideal time drive auto-built tests and time analysis;</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Difficulty: Easy, Medium or Hard. Ideal time in seconds. Marks: e.g. 3 and 1 (use 0 negative for type-in questions).</t>
+          <t>Concepts and Source let Guru find similar questions and previous-year questions for a student. Fill them whenever you can.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Image link: an https:// link to a chart or diagram for that question.</t>
+          <t>Difficulty Level: Very Easy, Easy, Medium, Hard or Very Hard (pick from the drop-down). Type: Single, Multiple or Numeric.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Upload both files in Admin → Tests → Upload tests (or Question bank → Add many to add questions without making a test).</t>
+          <t>Marks: e.g. 3 and 1 (use 0 negative for type-in questions). Correct Answer(s) is only needed when the Word file has no Answer: line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Instead of Topic and Subtopic you can use one Subject column with a path, e.g. "Quant (QA) &gt; Percentages &gt; Successive change".</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Hover over a heading in the Details sheet for help on that column.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Vendor-style test upload: D-range sets, pictures, optional option E, richer question details (#13)
- Word: Topic / Q.n) / a)-e) / Answer / Explanation; D.51-55) groups RC and DILR sets; pictures upload to the media table
- Option E only where a question has five options (bank form shows it on demand)
- Excel details: Type, Difficulty Level (Very Easy-Very Hard), Concepts, Source, Subject paths fill section > topic > subtopic
- Guru sees the student's weakest topics with unseen bank question counts
- Indexes for topic/level, subtopic and tag lookups; new templates


Claude-Session: https://claude.ai/code/session_01HobNgf1JPqeUaeRZMhfYbX

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/portal/public/question-details-template.xlsx
+++ b/portal/public/question-details-template.xlsx
@@ -44,7 +44,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3A8A"/>
+        <fgColor rgb="001E40AF"/>
       </patternFill>
     </fill>
   </fills>
@@ -63,7 +63,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -140,6 +140,76 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>DE Educare</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Same test name as the "Test:" line in Word. Can stay blank if the file has one test.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Fill if question numbers restart in each section.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Same number as in Word (Q.1) → 1).</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional if the Word file has Topic: lines (Word wins). Pick from the Topics sheet.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>The finer skill inside the topic, e.g. Successive discounts. Guru and practice sets use it.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Single (one answer), Multiple (several answers) or Numeric (type-in). Blank: worked out from the answer.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Very Easy, Easy, Medium, Hard or Very Hard.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>Time a well-prepared student should take, in seconds. Used in time analysis.</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>Comma-separated concepts or question patterns, e.g. ratio, weighted average. Guru uses them to find similar questions.</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>Original, or the paper, e.g. CAT 2023 Slot 2 (previous-year questions).</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <t>Only if the Word file has no Answer: line. a, or a,c for Multiple, or a number.</t>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <t>English, Hindi or Both.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -431,21 +501,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -461,7 +534,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Q No</t>
+          <t>Question Number</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -476,37 +549,52 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Difficulty</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Difficulty Level</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Ideal time (sec)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Marks if correct</t>
-        </is>
-      </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Negative marks</t>
+          <t>Marks</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Tags</t>
+          <t>Negative Marks</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>Concepts</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Image link</t>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Correct Answer(s)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Solution video</t>
         </is>
       </c>
     </row>
@@ -536,29 +624,40 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>120</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>3</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>1</v>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>rc</t>
-        </is>
-      </c>
       <c r="K2" t="inlineStr">
         <is>
+          <t>main idea, tone</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
           <t>Original</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -586,29 +685,40 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>Hard</t>
         </is>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>150</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>3</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>1</v>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>rc</t>
-        </is>
-      </c>
       <c r="K3" t="inlineStr">
         <is>
+          <t>inference</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
           <t>Original</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -618,47 +728,58 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>QA</t>
+          <t>VARC</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Percentages</t>
+          <t>Para Jumbles</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Successive change</t>
+          <t>Four-sentence jumble</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>60</v>
+          <t>Numeric</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Very Hard</t>
+        </is>
       </c>
       <c r="H4" t="n">
+        <v>120</v>
+      </c>
+      <c r="I4" t="n">
         <v>3</v>
       </c>
-      <c r="I4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>percent</t>
-        </is>
+      <c r="J4" t="n">
+        <v>0</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Original</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
+          <t>opening sentence, linkers</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>CAT 2023 Slot 2</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -672,7 +793,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -681,39 +802,50 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Basics</t>
+          <t>Successive change</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>Easy</t>
         </is>
       </c>
-      <c r="G5" t="n">
-        <v>45</v>
-      </c>
       <c r="H5" t="n">
+        <v>60</v>
+      </c>
+      <c r="I5" t="n">
         <v>3</v>
       </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>tita</t>
-        </is>
+      <c r="J5" t="n">
+        <v>1</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
+          <t>multiplying factors</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
           <t>Original</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAT Mock 2</t>
+          <t>CAT Mock 1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -722,47 +854,187 @@
         </is>
       </c>
       <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Percentages</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Percent of a number</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Numeric</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>30</v>
+      </c>
+      <c r="I6" t="n">
+        <v>3</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Bank PO Mock 1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
         <v>1</v>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Time, Speed &amp; Distance</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Relative speed</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Data Interpretation</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Bar graph</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G6" t="n">
-        <v>90</v>
-      </c>
-      <c r="H6" t="n">
-        <v>3</v>
-      </c>
-      <c r="I6" t="n">
+      <c r="H7" t="n">
+        <v>60</v>
+      </c>
+      <c r="I7" t="n">
         <v>1</v>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>CAT 2024 Slot 1</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
+      <c r="J7" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>difference, ranking</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Bank PO Mock 1</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Data Interpretation</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Bar graph</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>60</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="F2:F2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Easy,Medium,Hard"</formula1>
+  <dataValidations count="3">
+    <dataValidation sqref="F2:F5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Single,Multiple,Numeric"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Very Easy,Easy,Medium,Hard,Very Hard"</formula1>
+    </dataValidation>
+    <dataValidation sqref="N2:N5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"English,Hindi,Both"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -775,10 +1047,10 @@
   <dimension ref="A1:D73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2398,7 +2670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -2407,42 +2679,56 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>One row per question in the Word file. Test, Section and Q No must match the Word file (same test name, same section name, same question number).</t>
+          <t>One row per question in the Word file. Test, Section and Question Number must match the Word file.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>If question numbers restart in each section, fill Section. If they run through the whole test, Section can stay blank.</t>
+          <t>If question numbers restart in each section, fill Section. If they run through the whole test (like Q.51 … Q.55), Section can stay blank.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Topic: pick from the Topics sheet so reports and the auto test builder group questions correctly. A new topic is created if you type one that is not in the list.</t>
+          <t>Every column helps the question bank: Topic and Subtopic drive topic reports, SWOT and practice sets; Difficulty and Ideal time drive auto-built tests and time analysis;</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Difficulty: Easy, Medium or Hard. Ideal time in seconds. Marks: e.g. 3 and 1 (use 0 negative for type-in questions).</t>
+          <t>Concepts and Source let Guru find similar questions and previous-year questions for a student. Fill them whenever you can.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Image link: an https:// link to a chart or diagram for that question.</t>
+          <t>Difficulty Level: Very Easy, Easy, Medium, Hard or Very Hard (pick from the drop-down). Type: Single, Multiple or Numeric.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Upload both files in Admin → Tests → Upload tests (or Question bank → Add many to add questions without making a test).</t>
+          <t>Marks: e.g. 3 and 1 (use 0 negative for type-in questions). Correct Answer(s) is only needed when the Word file has no Answer: line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Instead of Topic and Subtopic you can use one Subject column with a path, e.g. "Quant (QA) &gt; Percentages &gt; Successive change".</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Hover over a heading in the Details sheet for help on that column.</t>
         </is>
       </c>
     </row>

</xml_diff>